<commit_message>
Processo de certificação: datas de transição da Global ACI
O fim da transição passa a 30/09/2029, e certificados novos só pela
edição de 2026 desde 31/03/2028, conforme o documento Global ACI-TECH-3-TR.
A cooperação internacional de acreditação passa a ser a Global ACI, que
substituiu o IAF e o ILAC em 2026. O painel encontra o próximo limite por
uma coluna auxiliar, sem MINIFS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Certificacao/Certificacao-modelo.xlsx
+++ b/Certificacao/Certificacao-modelo.xlsx
@@ -294,7 +294,7 @@
     <t xml:space="preserve">Transição</t>
   </si>
   <si>
-    <t xml:space="preserve">A ISO 9001:2026 foi publicada em 16/09/2026. O fim da transição vem preenchido com 16/09/2029, o prazo de três anos anunciado; confirme no comunicado da acreditação.</t>
+    <t xml:space="preserve">A ISO 9001:2026 foi publicada em 16/09/2026. O fim da transição vem preenchido com 30/09/2029, fixado pela Global ACI; desde 31/03/2028, certificados novos só pela edição de 2026. Confirme com o seu organismo.</t>
   </si>
   <si>
     <t xml:space="preserve">Exemplos</t>
@@ -1652,11 +1652,11 @@
         </c:ser>
         <c:gapWidth val="70"/>
         <c:overlap val="0"/>
-        <c:axId val="14226043"/>
-        <c:axId val="52100284"/>
+        <c:axId val="37895148"/>
+        <c:axId val="23941354"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="14226043"/>
+        <c:axId val="37895148"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1688,7 +1688,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52100284"/>
+        <c:crossAx val="23941354"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1696,7 +1696,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52100284"/>
+        <c:axId val="23941354"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1736,7 +1736,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14226043"/>
+        <c:crossAx val="37895148"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -2224,7 +2224,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="4" t="s">
         <v>54</v>
       </c>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="8" t="n">
-        <v>47377</v>
+        <v>47391</v>
       </c>
       <c r="F8" s="22" t="s">
         <v>107</v>
@@ -4860,16 +4860,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E7:E46 I7:K46" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="Em que auditoria a constatação foi feita" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D7:D46" type="list">
       <formula1>"Fase 1,Fase 2,Manutenção,Recertificação,Transição"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="NC maior, NC menor, oportunidade de melhoria ou ponto de atenção da fase 1" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F7:F46" type="list">
       <formula1>"NC maior,NC menor,Oportunidade de melhoria,Ponto de atenção da fase 1"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E7:E46 I7:K46" type="date">
+      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="35" t="n">
-        <v>47377</v>
+        <v>47391</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7258,7 +7258,7 @@
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="35" t="n">
-        <v>47377</v>
+        <v>47391</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="D44" s="24" t="n">
         <f aca="false">IF(OR($D$10="",$D$9&lt;&gt;"ISO 9001:2015"),"",MIN($D$12,$D$13))</f>
-        <v>47377</v>
+        <v>47391</v>
       </c>
       <c r="E44" s="41"/>
       <c r="F44" s="25" t="str">

</xml_diff>

<commit_message>
Leva 1: núcleo de auditoria, ficha em dia com a N23 e grau da não conformidade pelo critério
- Linha do tempo da ficha: auditoria 2026-03 com 3 NC menores.
- N05 marcada como superada por N23 em c4 e c6; regra N23 em PROIBIDO
  (Análise crítica).
- N24: o grau da não conformidade segue o critério de Auditoria, e não a
  repetição na amostra (Técnica, módulos 5 e 8 e exemplo 1; Certificação,
  definição da NC maior); regra N24 em PROIBIDO (Certificação).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Certificacao/Certificacao-modelo.xlsx
+++ b/Certificacao/Certificacao-modelo.xlsx
@@ -1652,11 +1652,11 @@
         </c:ser>
         <c:gapWidth val="70"/>
         <c:overlap val="0"/>
-        <c:axId val="17742"/>
-        <c:axId val="58749575"/>
+        <c:axId val="56692824"/>
+        <c:axId val="47123360"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="17742"/>
+        <c:axId val="56692824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1688,7 +1688,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58749575"/>
+        <c:crossAx val="47123360"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1696,7 +1696,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58749575"/>
+        <c:axId val="47123360"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1736,7 +1736,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17742"/>
+        <c:crossAx val="56692824"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -3318,12 +3318,12 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
+    <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="ISO 9001:2015 ou ISO 9001:2026" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D5" type="list">
+      <formula1>"ISO 9001:2015,ISO 9001:2026"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Digite uma data no formato dia/mês/ano." errorStyle="stop" errorTitle="Data inválida" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D6:D8 E13:E19" type="date">
       <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Escolha uma das opções da lista." errorStyle="stop" errorTitle="Valor inválido" operator="between" prompt="ISO 9001:2015 ou ISO 9001:2026" promptTitle="Opções" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D5" type="list">
-      <formula1>"ISO 9001:2015,ISO 9001:2026"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>